<commit_message>
Re-generate 2 qubit data with counts
</commit_message>
<xml_diff>
--- a/charts.xlsx
+++ b/charts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusedwards/Documents/Projects/EECE571F/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E9EA48-6E99-E246-8B3A-CB346369221C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FBFF894-2519-0A44-8226-BCE97142DCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30940" yWindow="100" windowWidth="28040" windowHeight="17440" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
   </bookViews>
@@ -714,6 +714,24 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$D$36:$D$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$A$36:$A$38</c:f>
@@ -768,6 +786,24 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$D$36:$D$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$B$36:$B$38</c:f>
@@ -822,6 +858,24 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$D$36:$D$38</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
               <c:f>Sheet1!$C$36:$C$38</c:f>
@@ -2658,7 +2712,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03013973-3BF3-2745-AF8D-DE558609215C}">
-  <dimension ref="A2:C38"/>
+  <dimension ref="A2:D38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -2716,12 +2770,12 @@
         <v>59845.974999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -2732,7 +2786,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>2115.1950000000002</v>
       </c>
@@ -2742,8 +2796,11 @@
       <c r="C36">
         <v>2280.0949999999998</v>
       </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>30218.309000000001</v>
       </c>
@@ -2753,8 +2810,11 @@
       <c r="C37">
         <v>31397.206999999999</v>
       </c>
+      <c r="D37">
+        <v>3</v>
+      </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>537522.75300000003</v>
       </c>
@@ -2763,6 +2823,9 @@
       </c>
       <c r="C38">
         <v>634056.321</v>
+      </c>
+      <c r="D38">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
More training data and direct comparison of Laplacian update with matmul
</commit_message>
<xml_diff>
--- a/charts.xlsx
+++ b/charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusedwards/Documents/Projects/EECE571F/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FBFF894-2519-0A44-8226-BCE97142DCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252C5038-4370-8048-BFE6-8D4358BE20BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-30940" yWindow="100" windowWidth="28040" windowHeight="17440" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
+    <workbookView xWindow="-71660" yWindow="-14800" windowWidth="47420" windowHeight="22900" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -47,8 +47,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Laplacian</t>
   </si>
@@ -70,18 +92,45 @@
   <si>
     <t>4 layers</t>
   </si>
+  <si>
+    <t>original approach</t>
+  </si>
+  <si>
+    <t>graph laplacian</t>
+  </si>
+  <si>
+    <t>32/46</t>
+  </si>
+  <si>
+    <t>27/46</t>
+  </si>
+  <si>
+    <t>2,2</t>
+  </si>
+  <si>
+    <t>2,3</t>
+  </si>
+  <si>
+    <t>20/46</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FFBCBEC4"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -104,8 +153,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2712,10 +2762,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03013973-3BF3-2745-AF8D-DE558609215C}">
-  <dimension ref="A2:D38"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A2:AQ79"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="19" max="19" width="20.33203125" customWidth="1"/>
+    <col min="20" max="20" width="34.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2726,7 +2780,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3">
       <c r="A3">
         <v>1097.01</v>
       </c>
@@ -2737,7 +2791,7 @@
         <v>114.73399999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3">
       <c r="A4">
         <v>14559.378000000001</v>
       </c>
@@ -2748,7 +2802,7 @@
         <v>1894.7059999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3">
       <c r="A5">
         <v>251362.774</v>
       </c>
@@ -2759,7 +2813,7 @@
         <v>43579.661</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3">
       <c r="A6">
         <v>717763.76</v>
       </c>
@@ -2770,12 +2824,161 @@
         <v>59845.974999999999</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="19:29">
+      <c r="S29" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC29" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="32" spans="19:29">
+      <c r="S32" t="s">
+        <v>7</v>
+      </c>
+      <c r="T32" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:43">
+      <c r="R33">
+        <v>1</v>
+      </c>
+      <c r="S33" s="1">
+        <v>1.43051147460937E-2</v>
+      </c>
+      <c r="T33" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="U33" t="b">
+        <f>T33&lt;S33</f>
+        <v>1</v>
+      </c>
+      <c r="V33">
+        <f>S33-T33</f>
+        <v>1.144409179687495E-2</v>
+      </c>
+      <c r="W33" cm="1">
+        <f t="array" ref="W33">IF(U33, V33, null)</f>
+        <v>1.144409179687495E-2</v>
+      </c>
+      <c r="X33">
+        <f>32/46</f>
+        <v>0.69565217391304346</v>
+      </c>
+      <c r="AA33">
+        <f>27/46</f>
+        <v>0.58695652173913049</v>
+      </c>
+      <c r="AC33" s="1">
+        <v>4.1007995605468701E-2</v>
+      </c>
+      <c r="AD33" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AE33" t="b">
+        <f>AD33&lt;AC33</f>
+        <v>1</v>
+      </c>
+      <c r="AF33">
+        <f>AC33-AD33</f>
+        <v>3.7908554077148389E-2</v>
+      </c>
+      <c r="AG33" cm="1">
+        <f t="array" ref="AG33">IF(AE33,AF33,null)</f>
+        <v>3.7908554077148389E-2</v>
+      </c>
+      <c r="AJ33">
+        <f>20/46</f>
+        <v>0.43478260869565216</v>
+      </c>
+      <c r="AL33" s="1">
+        <v>7.6055526733398396E-2</v>
+      </c>
+      <c r="AM33" s="1">
+        <v>5.9604644775390599E-3</v>
+      </c>
+      <c r="AN33" t="b">
+        <f>AM33&lt;AL33</f>
+        <v>1</v>
+      </c>
+      <c r="AO33">
+        <f>INT(AN33)</f>
+        <v>1</v>
+      </c>
+      <c r="AP33">
+        <f>AL33-AM33</f>
+        <v>7.0095062255859333E-2</v>
+      </c>
+      <c r="AQ33" cm="1">
+        <f t="array" ref="AQ33">IF(AN33,AP33,null)</f>
+        <v>7.0095062255859333E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:43">
       <c r="A34" t="s">
         <v>3</v>
       </c>
+      <c r="R34">
+        <v>2</v>
+      </c>
+      <c r="S34" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T34" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="U34" t="b">
+        <f t="shared" ref="U34:U78" si="0">T34&lt;S34</f>
+        <v>0</v>
+      </c>
+      <c r="V34">
+        <f t="shared" ref="V34:V78" si="1">S34-T34</f>
+        <v>-9.5367431640625E-4</v>
+      </c>
+      <c r="X34" t="s">
+        <v>9</v>
+      </c>
+      <c r="AA34" t="s">
+        <v>10</v>
+      </c>
+      <c r="AC34" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD34" s="1">
+        <v>1.5020370483398399E-2</v>
+      </c>
+      <c r="AE34" t="b">
+        <f t="shared" ref="AE34:AE78" si="2">AD34&lt;AC34</f>
+        <v>0</v>
+      </c>
+      <c r="AF34">
+        <f t="shared" ref="AF34:AF78" si="3">AC34-AD34</f>
+        <v>-1.192092895507809E-2</v>
+      </c>
+      <c r="AJ34" t="s">
+        <v>13</v>
+      </c>
+      <c r="AL34" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AM34" s="1">
+        <v>4.0769577026367097E-2</v>
+      </c>
+      <c r="AN34" t="b">
+        <f t="shared" ref="AN34:AN78" si="4">AM34&lt;AL34</f>
+        <v>0</v>
+      </c>
+      <c r="AO34">
+        <f t="shared" ref="AO34:AO78" si="5">INT(AN34)</f>
+        <v>0</v>
+      </c>
+      <c r="AP34">
+        <f t="shared" ref="AP34:AP78" si="6">AL34-AM34</f>
+        <v>-3.6716461181640535E-2</v>
+      </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:43">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -2785,8 +2988,69 @@
       <c r="C35" t="s">
         <v>6</v>
       </c>
+      <c r="R35">
+        <v>3</v>
+      </c>
+      <c r="S35" s="1">
+        <v>6.9141387939453099E-3</v>
+      </c>
+      <c r="T35" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U35" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V35">
+        <f t="shared" si="1"/>
+        <v>4.76837158203125E-3</v>
+      </c>
+      <c r="W35" cm="1">
+        <f t="array" ref="W35">IF(U35, V35, null)</f>
+        <v>4.76837158203125E-3</v>
+      </c>
+      <c r="AC35" s="1">
+        <v>1.2159347534179601E-2</v>
+      </c>
+      <c r="AD35" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AE35" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF35">
+        <f t="shared" si="3"/>
+        <v>9.0599060058592917E-3</v>
+      </c>
+      <c r="AG35" cm="1">
+        <f t="array" ref="AG35">IF(AE35,AF35,null)</f>
+        <v>9.0599060058592917E-3</v>
+      </c>
+      <c r="AL35" s="1">
+        <v>2.69412994384765E-2</v>
+      </c>
+      <c r="AM35" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AN35" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO35">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP35">
+        <f t="shared" si="6"/>
+        <v>2.2888183593749941E-2</v>
+      </c>
+      <c r="AQ35" cm="1">
+        <f t="array" ref="AQ35">IF(AN35,AP35,null)</f>
+        <v>2.2888183593749941E-2</v>
+      </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:43">
       <c r="A36">
         <v>2115.1950000000002</v>
       </c>
@@ -2799,8 +3063,61 @@
       <c r="D36">
         <v>2</v>
       </c>
+      <c r="R36">
+        <v>4</v>
+      </c>
+      <c r="S36" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T36" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U36" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V36">
+        <f t="shared" si="1"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AC36" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD36" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE36" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF36">
+        <f t="shared" si="3"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AG36" cm="1">
+        <f t="array" ref="AG36">IF(AE36,AF36,null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AL36" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AM36" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN36" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO36">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP36">
+        <f t="shared" si="6"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:43">
       <c r="A37">
         <v>30218.309000000001</v>
       </c>
@@ -2813,8 +3130,69 @@
       <c r="D37">
         <v>3</v>
       </c>
+      <c r="R37">
+        <v>5</v>
+      </c>
+      <c r="S37" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T37" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="U37" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V37">
+        <f t="shared" si="1"/>
+        <v>4.7683715820312999E-4</v>
+      </c>
+      <c r="W37" cm="1">
+        <f t="array" ref="W37">IF(U37, V37, null)</f>
+        <v>4.7683715820312999E-4</v>
+      </c>
+      <c r="AC37" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AD37" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AE37" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF37">
+        <f t="shared" si="3"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AG37" cm="1">
+        <f t="array" ref="AG37">IF(AE37,AF37,null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AL37" s="1">
+        <v>5.2452087402343698E-3</v>
+      </c>
+      <c r="AM37" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN37" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO37">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP37">
+        <f t="shared" si="6"/>
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AQ37" cm="1">
+        <f t="array" ref="AQ37">IF(AN37,AP37,null)</f>
+        <v>3.0994415283203099E-3</v>
+      </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:43">
       <c r="A38">
         <v>537522.75300000003</v>
       </c>
@@ -2826,6 +3204,2393 @@
       </c>
       <c r="D38">
         <v>4</v>
+      </c>
+      <c r="R38">
+        <v>6</v>
+      </c>
+      <c r="S38" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T38" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U38" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V38">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="W38" cm="1">
+        <f t="array" ref="W38">IF(U38, V38, null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AC38" s="1">
+        <v>5.0067901611328099E-3</v>
+      </c>
+      <c r="AD38" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE38" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF38">
+        <f t="shared" si="3"/>
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AG38" cm="1">
+        <f t="array" ref="AG38">IF(AE38,AF38,null)</f>
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AL38" s="1">
+        <v>7.1525573730468698E-3</v>
+      </c>
+      <c r="AM38" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="AN38" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO38">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP38">
+        <f t="shared" si="6"/>
+        <v>5.4836273193359401E-3</v>
+      </c>
+      <c r="AQ38" cm="1">
+        <f t="array" ref="AQ38">IF(AN38,AP38,null)</f>
+        <v>5.4836273193359401E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="1:43">
+      <c r="R39">
+        <v>7</v>
+      </c>
+      <c r="S39" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T39" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U39" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V39">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="W39" cm="1">
+        <f t="array" ref="W39">IF(U39, V39, null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AC39" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AD39" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AE39" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF39">
+        <f t="shared" si="3"/>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="AG39" cm="1">
+        <f t="array" ref="AG39">IF(AE39,AF39,null)</f>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="AL39" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AM39" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN39" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO39">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP39">
+        <f t="shared" si="6"/>
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AQ39" cm="1">
+        <f t="array" ref="AQ39">IF(AN39,AP39,null)</f>
+        <v>1.9073486328125E-3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:43">
+      <c r="R40">
+        <v>8</v>
+      </c>
+      <c r="S40" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T40" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U40" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V40">
+        <f t="shared" si="1"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AC40" s="1">
+        <v>3.814697265625E-3</v>
+      </c>
+      <c r="AD40" s="1">
+        <v>7.1525573730468696E-4</v>
+      </c>
+      <c r="AE40" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF40">
+        <f t="shared" si="3"/>
+        <v>3.0994415283203129E-3</v>
+      </c>
+      <c r="AG40" cm="1">
+        <f t="array" ref="AG40">IF(AE40,AF40,null)</f>
+        <v>3.0994415283203129E-3</v>
+      </c>
+      <c r="AL40" s="1">
+        <v>4.76837158203125E-3</v>
+      </c>
+      <c r="AM40" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN40" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO40">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP40">
+        <f t="shared" si="6"/>
+        <v>2.6226043701171901E-3</v>
+      </c>
+      <c r="AQ40" cm="1">
+        <f t="array" ref="AQ40">IF(AN40,AP40,null)</f>
+        <v>2.6226043701171901E-3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:43">
+      <c r="R41">
+        <v>9</v>
+      </c>
+      <c r="S41" s="1">
+        <v>5.9604644775390599E-3</v>
+      </c>
+      <c r="T41" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U41" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V41">
+        <f t="shared" si="1"/>
+        <v>3.814697265625E-3</v>
+      </c>
+      <c r="W41" cm="1">
+        <f t="array" ref="W41">IF(U41, V41, null)</f>
+        <v>3.814697265625E-3</v>
+      </c>
+      <c r="AC41" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AD41" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AE41" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF41">
+        <f t="shared" si="3"/>
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AG41" cm="1">
+        <f t="array" ref="AG41">IF(AE41,AF41,null)</f>
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AL41" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AM41" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN41" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO41">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP41">
+        <f t="shared" si="6"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:43">
+      <c r="R42">
+        <v>10</v>
+      </c>
+      <c r="S42" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T42" s="1">
+        <v>7.1525573730468696E-4</v>
+      </c>
+      <c r="U42" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V42">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078129E-3</v>
+      </c>
+      <c r="W42" cm="1">
+        <f t="array" ref="W42">IF(U42, V42, null)</f>
+        <v>1.1920928955078129E-3</v>
+      </c>
+      <c r="AC42" s="1">
+        <v>4.2915344238281198E-3</v>
+      </c>
+      <c r="AD42" s="1">
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AE42" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF42">
+        <f t="shared" si="3"/>
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AG42" cm="1">
+        <f t="array" ref="AG42">IF(AE42,AF42,null)</f>
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AL42" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM42" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AN42" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO42">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP42">
+        <f t="shared" si="6"/>
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AQ42" cm="1">
+        <f t="array" ref="AQ42">IF(AN42,AP42,null)</f>
+        <v>2.1457672119140599E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:43">
+      <c r="R43">
+        <v>11</v>
+      </c>
+      <c r="S43" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T43" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U43" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V43">
+        <f t="shared" si="1"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="W43" cm="1">
+        <f t="array" ref="W43">IF(U43, V43, null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AC43" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AD43" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AE43" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF43">
+        <f t="shared" si="3"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AG43" cm="1">
+        <f t="array" ref="AG43">IF(AE43,AF43,null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AL43" s="1">
+        <v>5.2452087402343698E-3</v>
+      </c>
+      <c r="AM43" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AN43" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO43">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP43">
+        <f t="shared" si="6"/>
+        <v>4.2915344238281198E-3</v>
+      </c>
+      <c r="AQ43" cm="1">
+        <f t="array" ref="AQ43">IF(AN43,AP43,null)</f>
+        <v>4.2915344238281198E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:43">
+      <c r="R44">
+        <v>12</v>
+      </c>
+      <c r="S44" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T44" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U44" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V44">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="W44" cm="1">
+        <f t="array" ref="W44">IF(U44, V44, null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AC44" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD44" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE44" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF44">
+        <f t="shared" si="3"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AG44" cm="1">
+        <f t="array" ref="AG44">IF(AE44,AF44,null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AL44" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AM44" s="1">
+        <v>6.1988830566406198E-3</v>
+      </c>
+      <c r="AN44" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO44">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP44">
+        <f t="shared" si="6"/>
+        <v>-3.3378601074218698E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:43">
+      <c r="R45">
+        <v>13</v>
+      </c>
+      <c r="S45" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T45" s="1">
+        <v>7.1525573730468696E-4</v>
+      </c>
+      <c r="U45" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V45">
+        <f t="shared" si="1"/>
+        <v>2.3841857910156228E-3</v>
+      </c>
+      <c r="W45" cm="1">
+        <f t="array" ref="W45">IF(U45, V45, null)</f>
+        <v>2.3841857910156228E-3</v>
+      </c>
+      <c r="AC45" s="1">
+        <v>5.0067901611328099E-3</v>
+      </c>
+      <c r="AD45" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE45" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF45">
+        <f t="shared" si="3"/>
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AG45" cm="1">
+        <f t="array" ref="AG45">IF(AE45,AF45,null)</f>
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AL45" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM45" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AN45" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO45">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP45">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:43">
+      <c r="R46">
+        <v>14</v>
+      </c>
+      <c r="S46" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="T46" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U46" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V46">
+        <f t="shared" si="1"/>
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="W46" cm="1">
+        <f t="array" ref="W46">IF(U46, V46, null)</f>
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AC46" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AD46" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE46" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF46">
+        <f t="shared" si="3"/>
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AG46" cm="1">
+        <f t="array" ref="AG46">IF(AE46,AF46,null)</f>
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AL46" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM46" s="1">
+        <v>6.9141387939453099E-3</v>
+      </c>
+      <c r="AN46" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO46">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP46">
+        <f t="shared" si="6"/>
+        <v>-3.814697265625E-3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:43">
+      <c r="R47">
+        <v>15</v>
+      </c>
+      <c r="S47" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T47" s="1">
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="U47" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V47">
+        <f t="shared" si="1"/>
+        <v>7.152557373046901E-4</v>
+      </c>
+      <c r="W47" cm="1">
+        <f t="array" ref="W47">IF(U47, V47, null)</f>
+        <v>7.152557373046901E-4</v>
+      </c>
+      <c r="AC47" s="1">
+        <v>4.2915344238281198E-3</v>
+      </c>
+      <c r="AD47" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE47" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF47">
+        <f t="shared" si="3"/>
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AG47" cm="1">
+        <f t="array" ref="AG47">IF(AE47,AF47,null)</f>
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AL47" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM47" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AN47" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO47">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP47">
+        <f t="shared" si="6"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AQ47" cm="1">
+        <f t="array" ref="AQ47">IF(AN47,AP47,null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:43">
+      <c r="R48">
+        <v>16</v>
+      </c>
+      <c r="S48" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T48" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U48" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V48">
+        <f t="shared" si="1"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AC48" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AD48" s="1">
+        <v>3.814697265625E-3</v>
+      </c>
+      <c r="AE48" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF48">
+        <f t="shared" si="3"/>
+        <v>-1.6689300537109401E-3</v>
+      </c>
+      <c r="AL48" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AM48" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AN48" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO48">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP48">
+        <f t="shared" si="6"/>
+        <v>-9.5367431640625E-4</v>
+      </c>
+    </row>
+    <row r="49" spans="18:43">
+      <c r="R49">
+        <v>17</v>
+      </c>
+      <c r="S49" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T49" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U49" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V49">
+        <f t="shared" si="1"/>
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="W49" cm="1">
+        <f t="array" ref="W49">IF(U49, V49, null)</f>
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AC49" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AD49" s="1">
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AE49" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF49">
+        <f t="shared" si="3"/>
+        <v>1.6689300537109401E-3</v>
+      </c>
+      <c r="AG49" cm="1">
+        <f t="array" ref="AG49">IF(AE49,AF49,null)</f>
+        <v>1.6689300537109401E-3</v>
+      </c>
+      <c r="AL49" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM49" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AN49" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO49">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP49">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="18:43">
+      <c r="R50">
+        <v>18</v>
+      </c>
+      <c r="S50" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T50" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U50" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V50">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC50" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD50" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AE50" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF50">
+        <f t="shared" si="3"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AG50" cm="1">
+        <f t="array" ref="AG50">IF(AE50,AF50,null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AL50" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AM50" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AN50" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO50">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP50">
+        <f t="shared" si="6"/>
+        <v>-1.1920928955078099E-3</v>
+      </c>
+    </row>
+    <row r="51" spans="18:43">
+      <c r="R51">
+        <v>19</v>
+      </c>
+      <c r="S51" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="T51" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U51" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V51">
+        <f t="shared" si="1"/>
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="W51" cm="1">
+        <f t="array" ref="W51">IF(U51, V51, null)</f>
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AC51" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AD51" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE51" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF51">
+        <f t="shared" si="3"/>
+        <v>7.152557373046901E-4</v>
+      </c>
+      <c r="AG51" cm="1">
+        <f t="array" ref="AG51">IF(AE51,AF51,null)</f>
+        <v>7.152557373046901E-4</v>
+      </c>
+      <c r="AL51" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM51" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN51" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO51">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP51">
+        <f t="shared" si="6"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AQ51" cm="1">
+        <f t="array" ref="AQ51">IF(AN51,AP51,null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+    </row>
+    <row r="52" spans="18:43">
+      <c r="R52">
+        <v>20</v>
+      </c>
+      <c r="S52" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T52" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U52" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V52">
+        <f t="shared" si="1"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="W52" cm="1">
+        <f t="array" ref="W52">IF(U52, V52, null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AC52" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD52" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AE52" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF52">
+        <f t="shared" si="3"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AG52" cm="1">
+        <f t="array" ref="AG52">IF(AE52,AF52,null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AL52" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AM52" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AN52" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO52">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP52">
+        <f t="shared" si="6"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AQ52" cm="1">
+        <f t="array" ref="AQ52">IF(AN52,AP52,null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+    </row>
+    <row r="53" spans="18:43">
+      <c r="R53">
+        <v>21</v>
+      </c>
+      <c r="S53" s="1">
+        <v>2.6226043701171801E-3</v>
+      </c>
+      <c r="T53" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U53" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V53">
+        <f t="shared" si="1"/>
+        <v>7.1525573730468013E-4</v>
+      </c>
+      <c r="W53" cm="1">
+        <f t="array" ref="W53">IF(U53, V53, null)</f>
+        <v>7.1525573730468013E-4</v>
+      </c>
+      <c r="AC53" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD53" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="AE53" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF53">
+        <f t="shared" si="3"/>
+        <v>2.3841857910157009E-4</v>
+      </c>
+      <c r="AG53" cm="1">
+        <f t="array" ref="AG53">IF(AE53,AF53,null)</f>
+        <v>2.3841857910157009E-4</v>
+      </c>
+      <c r="AL53" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AM53" s="1">
+        <v>5.0067901611328099E-3</v>
+      </c>
+      <c r="AN53" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO53">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP53">
+        <f t="shared" si="6"/>
+        <v>-2.86102294921875E-3</v>
+      </c>
+    </row>
+    <row r="54" spans="18:43">
+      <c r="R54">
+        <v>22</v>
+      </c>
+      <c r="S54" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T54" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U54" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V54">
+        <f t="shared" si="1"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="W54" cm="1">
+        <f t="array" ref="W54">IF(U54, V54, null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AC54" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD54" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AE54" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF54">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AL54" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AM54" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN54" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO54">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP54">
+        <f t="shared" si="6"/>
+        <v>7.152557373046901E-4</v>
+      </c>
+      <c r="AQ54" cm="1">
+        <f t="array" ref="AQ54">IF(AN54,AP54,null)</f>
+        <v>7.152557373046901E-4</v>
+      </c>
+    </row>
+    <row r="55" spans="18:43">
+      <c r="R55">
+        <v>23</v>
+      </c>
+      <c r="S55" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T55" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U55" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V55">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC55" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD55" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE55" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF55">
+        <f t="shared" si="3"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AL55" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM55" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="AN55" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO55">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP55">
+        <f t="shared" si="6"/>
+        <v>1.43051147460938E-3</v>
+      </c>
+      <c r="AQ55" cm="1">
+        <f t="array" ref="AQ55">IF(AN55,AP55,null)</f>
+        <v>1.43051147460938E-3</v>
+      </c>
+    </row>
+    <row r="56" spans="18:43">
+      <c r="R56">
+        <v>24</v>
+      </c>
+      <c r="S56" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T56" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U56" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V56">
+        <f t="shared" si="1"/>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="W56" cm="1">
+        <f t="array" ref="W56">IF(U56, V56, null)</f>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="AC56" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AD56" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AE56" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF56">
+        <f t="shared" si="3"/>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="AG56" cm="1">
+        <f t="array" ref="AG56">IF(AE56,AF56,null)</f>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="AL56" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="AM56" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN56" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO56">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP56">
+        <f t="shared" si="6"/>
+        <v>-4.7683715820312999E-4</v>
+      </c>
+    </row>
+    <row r="57" spans="18:43">
+      <c r="R57">
+        <v>25</v>
+      </c>
+      <c r="S57" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T57" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U57" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V57">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="W57" cm="1">
+        <f t="array" ref="W57">IF(U57, V57, null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AC57" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD57" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AE57" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF57">
+        <f t="shared" si="3"/>
+        <v>-1.1920928955078099E-3</v>
+      </c>
+      <c r="AL57" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM57" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AN57" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO57">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP57">
+        <f t="shared" si="6"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AQ57" cm="1">
+        <f t="array" ref="AQ57">IF(AN57,AP57,null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+    </row>
+    <row r="58" spans="18:43">
+      <c r="R58">
+        <v>26</v>
+      </c>
+      <c r="S58" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T58" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U58" t="b">
+        <f>T58&lt;S58</f>
+        <v>0</v>
+      </c>
+      <c r="V58">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC58" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AD58" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AE58" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF58">
+        <f t="shared" si="3"/>
+        <v>-7.152557373046901E-4</v>
+      </c>
+      <c r="AL58" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AM58" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AN58" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO58">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP58">
+        <f t="shared" si="6"/>
+        <v>-1.1920928955078099E-3</v>
+      </c>
+    </row>
+    <row r="59" spans="18:43">
+      <c r="R59">
+        <v>27</v>
+      </c>
+      <c r="S59" s="1">
+        <v>6.9141387939453099E-3</v>
+      </c>
+      <c r="T59" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U59" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V59">
+        <f t="shared" si="1"/>
+        <v>4.76837158203125E-3</v>
+      </c>
+      <c r="W59" cm="1">
+        <f t="array" ref="W59">IF(U59, V59, null)</f>
+        <v>4.76837158203125E-3</v>
+      </c>
+      <c r="AC59" s="1">
+        <v>1.52587890625E-2</v>
+      </c>
+      <c r="AD59" s="1">
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AE59" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF59">
+        <f t="shared" si="3"/>
+        <v>1.4066696166992191E-2</v>
+      </c>
+      <c r="AG59" cm="1">
+        <f t="array" ref="AG59">IF(AE59,AF59,null)</f>
+        <v>1.4066696166992191E-2</v>
+      </c>
+      <c r="AL59" s="1">
+        <v>2.8133392333984299E-2</v>
+      </c>
+      <c r="AM59" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN59" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO59">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP59">
+        <f t="shared" si="6"/>
+        <v>2.598762512207024E-2</v>
+      </c>
+      <c r="AQ59" cm="1">
+        <f t="array" ref="AQ59">IF(AN59,AP59,null)</f>
+        <v>2.598762512207024E-2</v>
+      </c>
+    </row>
+    <row r="60" spans="18:43">
+      <c r="R60">
+        <v>28</v>
+      </c>
+      <c r="S60" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T60" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U60" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V60">
+        <f t="shared" si="1"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AC60" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD60" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE60" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF60">
+        <f t="shared" si="3"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AL60" s="1">
+        <v>5.0067901611328099E-3</v>
+      </c>
+      <c r="AM60" s="1">
+        <v>2.6226043701171801E-3</v>
+      </c>
+      <c r="AN60" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO60">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP60">
+        <f t="shared" si="6"/>
+        <v>2.3841857910156298E-3</v>
+      </c>
+      <c r="AQ60" cm="1">
+        <f t="array" ref="AQ60">IF(AN60,AP60,null)</f>
+        <v>2.3841857910156298E-3</v>
+      </c>
+    </row>
+    <row r="61" spans="18:43">
+      <c r="R61">
+        <v>29</v>
+      </c>
+      <c r="S61" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="T61" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="U61" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V61">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078201E-3</v>
+      </c>
+      <c r="W61" cm="1">
+        <f t="array" ref="W61">IF(U61, V61, null)</f>
+        <v>1.1920928955078201E-3</v>
+      </c>
+      <c r="AC61" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD61" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AE61" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF61">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AL61" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AM61" s="1">
+        <v>5.9604644775390599E-3</v>
+      </c>
+      <c r="AN61" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO61">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP61">
+        <f t="shared" si="6"/>
+        <v>-3.0994415283203099E-3</v>
+      </c>
+    </row>
+    <row r="62" spans="18:43">
+      <c r="R62">
+        <v>30</v>
+      </c>
+      <c r="S62" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T62" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U62" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V62">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="W62" cm="1">
+        <f t="array" ref="W62">IF(U62, V62, null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AC62" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD62" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE62" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF62">
+        <f t="shared" si="3"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AG62" cm="1">
+        <f t="array" ref="AG62">IF(AE62,AF62,null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AL62" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AM62" s="1">
+        <v>1.1920928955078101E-2</v>
+      </c>
+      <c r="AN62" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO62">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP62">
+        <f t="shared" si="6"/>
+        <v>-1.0013580322265601E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="18:43">
+      <c r="R63">
+        <v>31</v>
+      </c>
+      <c r="S63" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="T63" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U63" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V63">
+        <f t="shared" si="1"/>
+        <v>7.1525573730467991E-4</v>
+      </c>
+      <c r="W63" cm="1">
+        <f t="array" ref="W63">IF(U63, V63, null)</f>
+        <v>7.1525573730467991E-4</v>
+      </c>
+      <c r="AC63" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="AD63" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AE63" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF63">
+        <f t="shared" si="3"/>
+        <v>-2.3841857910157009E-4</v>
+      </c>
+      <c r="AL63" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AM63" s="1">
+        <v>7.8678131103515608E-3</v>
+      </c>
+      <c r="AN63" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO63">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP63">
+        <f t="shared" si="6"/>
+        <v>-5.7220458984375009E-3</v>
+      </c>
+    </row>
+    <row r="64" spans="18:43">
+      <c r="R64">
+        <v>32</v>
+      </c>
+      <c r="S64" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T64" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U64" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V64">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="W64" cm="1">
+        <f t="array" ref="W64">IF(U64, V64, null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AC64" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD64" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AE64" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF64">
+        <f t="shared" si="3"/>
+        <v>-9.5367431640625E-4</v>
+      </c>
+      <c r="AL64" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM64" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AN64" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO64">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP64">
+        <f t="shared" si="6"/>
+        <v>-9.5367431640625E-4</v>
+      </c>
+    </row>
+    <row r="65" spans="18:43">
+      <c r="R65">
+        <v>33</v>
+      </c>
+      <c r="S65" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="T65" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U65" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V65">
+        <f t="shared" si="1"/>
+        <v>-1.1920928955078099E-3</v>
+      </c>
+      <c r="AC65" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AD65" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AE65" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF65">
+        <f t="shared" si="3"/>
+        <v>-1.9073486328125E-3</v>
+      </c>
+      <c r="AL65" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AM65" s="1">
+        <v>5.0067901611328099E-3</v>
+      </c>
+      <c r="AN65" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO65">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP65">
+        <f t="shared" si="6"/>
+        <v>-3.0994415283203099E-3</v>
+      </c>
+    </row>
+    <row r="66" spans="18:43">
+      <c r="R66">
+        <v>34</v>
+      </c>
+      <c r="S66" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T66" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="U66" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V66">
+        <f t="shared" si="1"/>
+        <v>1.43051147460938E-3</v>
+      </c>
+      <c r="W66" cm="1">
+        <f t="array" ref="W66">IF(U66, V66, null)</f>
+        <v>1.43051147460938E-3</v>
+      </c>
+      <c r="AC66" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD66" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AE66" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF66">
+        <f t="shared" si="3"/>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="AG66" cm="1">
+        <f t="array" ref="AG66">IF(AE66,AF66,null)</f>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="AL66" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM66" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN66" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO66">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP66">
+        <f t="shared" si="6"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AQ66" cm="1">
+        <f t="array" ref="AQ66">IF(AN66,AP66,null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+    </row>
+    <row r="67" spans="18:43">
+      <c r="R67">
+        <v>35</v>
+      </c>
+      <c r="S67" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T67" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U67" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V67">
+        <f t="shared" si="1"/>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="W67" cm="1">
+        <f t="array" ref="W67">IF(U67, V67, null)</f>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="AC67" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD67" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AE67" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF67">
+        <f t="shared" si="3"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AG67" cm="1">
+        <f t="array" ref="AG67">IF(AE67,AF67,null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AL67" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM67" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AN67" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO67">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP67">
+        <f t="shared" si="6"/>
+        <v>-9.5367431640625E-4</v>
+      </c>
+    </row>
+    <row r="68" spans="18:43">
+      <c r="R68">
+        <v>36</v>
+      </c>
+      <c r="S68" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T68" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U68" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V68">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC68" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD68" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AE68" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF68">
+        <f t="shared" si="3"/>
+        <v>-9.5367431640625E-4</v>
+      </c>
+      <c r="AL68" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AM68" s="1">
+        <v>5.0067901611328099E-3</v>
+      </c>
+      <c r="AN68" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO68">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP68">
+        <f t="shared" si="6"/>
+        <v>-2.1457672119140599E-3</v>
+      </c>
+    </row>
+    <row r="69" spans="18:43">
+      <c r="R69">
+        <v>37</v>
+      </c>
+      <c r="S69" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T69" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U69" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V69">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC69" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AD69" s="1">
+        <v>4.0531158447265599E-3</v>
+      </c>
+      <c r="AE69" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF69">
+        <f t="shared" si="3"/>
+        <v>-1.9073486328125E-3</v>
+      </c>
+      <c r="AL69" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM69" s="1">
+        <v>8.3446502685546806E-3</v>
+      </c>
+      <c r="AN69" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO69">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP69">
+        <f t="shared" si="6"/>
+        <v>-5.2452087402343707E-3</v>
+      </c>
+    </row>
+    <row r="70" spans="18:43">
+      <c r="R70">
+        <v>38</v>
+      </c>
+      <c r="S70" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T70" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="U70" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V70">
+        <f t="shared" si="1"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AC70" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD70" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AE70" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF70">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AL70" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="AM70" s="1">
+        <v>6.9141387939453099E-3</v>
+      </c>
+      <c r="AN70" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO70">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP70">
+        <f t="shared" si="6"/>
+        <v>-5.2452087402343802E-3</v>
+      </c>
+    </row>
+    <row r="71" spans="18:43">
+      <c r="R71">
+        <v>39</v>
+      </c>
+      <c r="S71" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="T71" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U71" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V71">
+        <f t="shared" si="1"/>
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="W71" cm="1">
+        <f t="array" ref="W71">IF(U71, V71, null)</f>
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AC71" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD71" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE71" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF71">
+        <f t="shared" si="3"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AG71" cm="1">
+        <f t="array" ref="AG71">IF(AE71,AF71,null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AL71" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AM71" s="1">
+        <v>5.2452087402343698E-3</v>
+      </c>
+      <c r="AN71" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO71">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP71">
+        <f t="shared" si="6"/>
+        <v>-3.0994415283203099E-3</v>
+      </c>
+    </row>
+    <row r="72" spans="18:43">
+      <c r="R72">
+        <v>40</v>
+      </c>
+      <c r="S72" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T72" s="1">
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="U72" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V72">
+        <f t="shared" si="1"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="W72" cm="1">
+        <f t="array" ref="W72">IF(U72, V72, null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AC72" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD72" s="1">
+        <v>7.1525573730468696E-4</v>
+      </c>
+      <c r="AE72" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF72">
+        <f t="shared" si="3"/>
+        <v>2.3841857910156228E-3</v>
+      </c>
+      <c r="AG72" cm="1">
+        <f t="array" ref="AG72">IF(AE72,AF72,null)</f>
+        <v>2.3841857910156228E-3</v>
+      </c>
+      <c r="AL72" s="1">
+        <v>2.6226043701171801E-3</v>
+      </c>
+      <c r="AM72" s="1">
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AN72" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO72">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP72">
+        <f t="shared" si="6"/>
+        <v>1.4305114746093702E-3</v>
+      </c>
+      <c r="AQ72" cm="1">
+        <f t="array" ref="AQ72">IF(AN72,AP72,null)</f>
+        <v>1.4305114746093702E-3</v>
+      </c>
+    </row>
+    <row r="73" spans="18:43">
+      <c r="R73">
+        <v>41</v>
+      </c>
+      <c r="S73" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T73" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U73" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V73">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="W73" cm="1">
+        <f t="array" ref="W73">IF(U73, V73, null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AC73" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD73" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AE73" t="b">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="AF73">
+        <f t="shared" si="3"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AG73" cm="1">
+        <f t="array" ref="AG73">IF(AE73,AF73,null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AL73" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AM73" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AN73" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO73">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP73">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="18:43">
+      <c r="R74">
+        <v>42</v>
+      </c>
+      <c r="S74" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T74" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U74" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V74">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC74" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AD74" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE74" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF74">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AL74" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="AM74" s="1">
+        <v>1.6689300537109299E-3</v>
+      </c>
+      <c r="AN74" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO74">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP74">
+        <f t="shared" si="6"/>
+        <v>1.1920928955078201E-3</v>
+      </c>
+      <c r="AQ74" cm="1">
+        <f t="array" ref="AQ74">IF(AN74,AP74,null)</f>
+        <v>1.1920928955078201E-3</v>
+      </c>
+    </row>
+    <row r="75" spans="18:43">
+      <c r="R75">
+        <v>43</v>
+      </c>
+      <c r="S75" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="T75" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U75" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V75">
+        <f t="shared" si="1"/>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="W75" cm="1">
+        <f t="array" ref="W75">IF(U75, V75, null)</f>
+        <v>1.1920928955078099E-3</v>
+      </c>
+      <c r="AC75" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD75" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE75" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF75">
+        <f t="shared" si="3"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AL75" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AM75" s="1">
+        <v>5.0067901611328099E-3</v>
+      </c>
+      <c r="AN75" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO75">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP75">
+        <f t="shared" si="6"/>
+        <v>-1.9073486328125E-3</v>
+      </c>
+    </row>
+    <row r="76" spans="18:43">
+      <c r="R76">
+        <v>44</v>
+      </c>
+      <c r="S76" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="T76" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="U76" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V76">
+        <f t="shared" si="1"/>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="W76" cm="1">
+        <f t="array" ref="W76">IF(U76, V76, null)</f>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="AC76" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD76" s="1">
+        <v>6.9141387939453099E-3</v>
+      </c>
+      <c r="AE76" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF76">
+        <f t="shared" si="3"/>
+        <v>-5.0067901611328099E-3</v>
+      </c>
+      <c r="AL76" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AM76" s="1">
+        <v>1.3113021850585899E-2</v>
+      </c>
+      <c r="AN76" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO76">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP76">
+        <f t="shared" si="6"/>
+        <v>-1.096725463867184E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="18:43">
+      <c r="R77">
+        <v>45</v>
+      </c>
+      <c r="S77" s="1">
+        <v>2.86102294921875E-3</v>
+      </c>
+      <c r="T77" s="1">
+        <v>4.2915344238281198E-3</v>
+      </c>
+      <c r="U77" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V77">
+        <f t="shared" si="1"/>
+        <v>-1.4305114746093698E-3</v>
+      </c>
+      <c r="AC77" s="1">
+        <v>3.0994415283203099E-3</v>
+      </c>
+      <c r="AD77" s="1">
+        <v>6.1988830566406198E-3</v>
+      </c>
+      <c r="AE77" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF77">
+        <f t="shared" si="3"/>
+        <v>-3.0994415283203099E-3</v>
+      </c>
+      <c r="AL77" s="1">
+        <v>3.814697265625E-3</v>
+      </c>
+      <c r="AM77" s="1">
+        <v>1.0013580322265601E-2</v>
+      </c>
+      <c r="AN77" t="b">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AO77">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP77">
+        <f t="shared" si="6"/>
+        <v>-6.1988830566406007E-3</v>
+      </c>
+    </row>
+    <row r="78" spans="18:43">
+      <c r="R78">
+        <v>46</v>
+      </c>
+      <c r="S78" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T78" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U78" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="V78">
+        <f t="shared" si="1"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="W78" cm="1">
+        <f t="array" ref="W78">IF(U78, V78, null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AC78" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD78" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE78" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF78">
+        <f t="shared" si="3"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AL78" s="1">
+        <v>6.1988830566406198E-3</v>
+      </c>
+      <c r="AM78" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AN78" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO78">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP78">
+        <f t="shared" si="6"/>
+        <v>4.2915344238281198E-3</v>
+      </c>
+      <c r="AQ78" cm="1">
+        <f t="array" ref="AQ78">IF(AN78,AP78,null)</f>
+        <v>4.2915344238281198E-3</v>
+      </c>
+    </row>
+    <row r="79" spans="18:43">
+      <c r="V79">
+        <f>AVERAGE(V33:V78)</f>
+        <v>1.1247137318486744E-3</v>
+      </c>
+      <c r="W79">
+        <f>AVERAGE(W33:W78)</f>
+        <v>1.7657876014709455E-3</v>
+      </c>
+      <c r="AG79">
+        <f>AVERAGE(AG33:AG75)</f>
+        <v>3.5674483687789305E-3</v>
+      </c>
+      <c r="AO79">
+        <f>SUM(AO33:AO78)</f>
+        <v>20</v>
+      </c>
+      <c r="AQ79">
+        <f>AVERAGE(AQ33:AQ78)</f>
+        <v>7.7605247497558507E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Convert usages of np to jnp
</commit_message>
<xml_diff>
--- a/charts.xlsx
+++ b/charts.xlsx
@@ -8,24 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusedwards/Documents/Projects/EECE571F/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252C5038-4370-8048-BFE6-8D4358BE20BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B456CA-2306-5A45-880F-C8CB823F22AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-71660" yWindow="-14800" windowWidth="47420" windowHeight="22900" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
+    <workbookView xWindow="-36300" yWindow="-15240" windowWidth="31120" windowHeight="23200" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v2.0" hidden="1">Sheet1!$A$1:$C$35</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">Sheet1!$A$36:$C$36</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">Sheet1!$A$37:$C$37</definedName>
-    <definedName name="_xlchart.v2.3" hidden="1">Sheet1!$A$38:$C$38</definedName>
-    <definedName name="_xlchart.v2.4" hidden="1">Sheet1!$A$34:$A$35</definedName>
-    <definedName name="_xlchart.v2.5" hidden="1">Sheet1!$A$36:$A$38</definedName>
-    <definedName name="_xlchart.v2.6" hidden="1">Sheet1!$B$34:$B$35</definedName>
-    <definedName name="_xlchart.v2.7" hidden="1">Sheet1!$B$36:$B$38</definedName>
-    <definedName name="_xlchart.v2.8" hidden="1">Sheet1!$C$34:$C$35</definedName>
-    <definedName name="_xlchart.v2.9" hidden="1">Sheet1!$C$36:$C$38</definedName>
+    <definedName name="_xlchart.v2.0" hidden="1">Sheet1!$A$66</definedName>
+    <definedName name="_xlchart.v2.1" hidden="1">Sheet1!$A$67:$A$70</definedName>
+    <definedName name="_xlchart.v2.2" hidden="1">Sheet1!$B$66</definedName>
+    <definedName name="_xlchart.v2.3" hidden="1">Sheet1!$B$67:$B$70</definedName>
+    <definedName name="_xlchart.v2.4" hidden="1">Sheet1!$C$66</definedName>
+    <definedName name="_xlchart.v2.5" hidden="1">Sheet1!$C$67:$C$70</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -70,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>Laplacian</t>
   </si>
@@ -112,6 +108,18 @@
   </si>
   <si>
     <t>20/46</t>
+  </si>
+  <si>
+    <t>Direct comparison</t>
+  </si>
+  <si>
+    <t>Density Matrix</t>
+  </si>
+  <si>
+    <t>Layers</t>
+  </si>
+  <si>
+    <t>Difference</t>
   </si>
 </sst>
 </file>
@@ -208,7 +216,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Performance Scaling</a:t>
+              <a:t>2-Qubit Performance Scaling</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -274,12 +282,30 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$D$3:$D$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$A$3:$A$6</c:f>
+              <c:f>Sheet1!$A$3:$A$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>1097.01</c:v>
                 </c:pt>
@@ -288,9 +314,6 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>251362.774</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>717763.76</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -328,12 +351,30 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$D$3:$D$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$3:$B$6</c:f>
+              <c:f>Sheet1!$B$3:$B$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>253.64699999999999</c:v>
                 </c:pt>
@@ -342,9 +383,6 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>79616.144</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>109594.58100000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -382,12 +420,30 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$D$3:$D$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$3:$C$6</c:f>
+              <c:f>Sheet1!$C$3:$C$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="4"/>
+                <c:ptCount val="3"/>
                 <c:pt idx="0">
                   <c:v>114.73399999999999</c:v>
                 </c:pt>
@@ -396,9 +452,6 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>43579.661</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>59845.974999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -429,6 +482,61 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Layers</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1256,6 +1364,524 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>2-Qubit Ab Initio Comparison</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$A$66</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Laplacian</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$D$67:$D$69</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$A$67:$A$69</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>120.083</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1902.8409999999999</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30158.742999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FEAE-BD41-97F2-9234F09370B4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$B$66</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Density Matrix</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Sheet1!$D$67:$D$69</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$67:$B$69</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>213.60900000000001</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3296.7440000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>51611.423000000003</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-FEAE-BD41-97F2-9234F09370B4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="351043440"/>
+        <c:axId val="351040288"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="351043440"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Layers</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="351040288"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="351040288"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>milliseconds</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="351043440"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -1336,6 +1962,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
@@ -1853,6 +2519,522 @@
 </file>
 
 <file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2437,6 +3619,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>692150</xdr:colOff>
+      <xdr:row>71</xdr:row>
+      <xdr:rowOff>120650</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>139700</xdr:colOff>
+      <xdr:row>102</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA100448-034B-15E1-4BCB-86E09F40582E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2762,14 +3980,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03013973-3BF3-2745-AF8D-DE558609215C}">
-  <dimension ref="A2:AQ79"/>
+  <dimension ref="A2:AQ89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="19" max="19" width="20.33203125" customWidth="1"/>
     <col min="20" max="20" width="34.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2780,7 +3998,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3">
         <v>1097.01</v>
       </c>
@@ -2790,8 +4008,11 @@
       <c r="C3">
         <v>114.73399999999999</v>
       </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>14559.378000000001</v>
       </c>
@@ -2801,8 +4022,11 @@
       <c r="C4">
         <v>1894.7059999999999</v>
       </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>251362.774</v>
       </c>
@@ -2812,8 +4036,11 @@
       <c r="C5">
         <v>43579.661</v>
       </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>717763.76</v>
       </c>
@@ -2822,6 +4049,9 @@
       </c>
       <c r="C6">
         <v>59845.974999999999</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="19:29">
@@ -4789,7 +6019,10 @@
         <v>-9.5367431640625E-4</v>
       </c>
     </row>
-    <row r="65" spans="18:43">
+    <row r="65" spans="1:43">
+      <c r="A65" t="s">
+        <v>14</v>
+      </c>
       <c r="R65">
         <v>33</v>
       </c>
@@ -4840,7 +6073,19 @@
         <v>-3.0994415283203099E-3</v>
       </c>
     </row>
-    <row r="66" spans="18:43">
+    <row r="66" spans="1:43">
+      <c r="A66" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" t="s">
+        <v>15</v>
+      </c>
+      <c r="C66" t="s">
+        <v>17</v>
+      </c>
+      <c r="D66" t="s">
+        <v>16</v>
+      </c>
       <c r="R66">
         <v>34</v>
       </c>
@@ -4903,7 +6148,30 @@
         <v>9.5367431640625E-4</v>
       </c>
     </row>
-    <row r="67" spans="18:43">
+    <row r="67" spans="1:43">
+      <c r="A67">
+        <v>120.083</v>
+      </c>
+      <c r="B67">
+        <v>213.60900000000001</v>
+      </c>
+      <c r="C67">
+        <f>B67-A67</f>
+        <v>93.52600000000001</v>
+      </c>
+      <c r="D67">
+        <v>2</v>
+      </c>
+      <c r="F67" cm="1">
+        <f t="array" ref="F67:H67">LINEST(C67:C69,D67:D69^{1,2})</f>
+        <v>9379.200000000008</v>
+      </c>
+      <c r="G67">
+        <v>-45595.623000000043</v>
+      </c>
+      <c r="H67">
+        <v>53767.972000000053</v>
+      </c>
       <c r="R67">
         <v>35</v>
       </c>
@@ -4962,7 +6230,27 @@
         <v>-9.5367431640625E-4</v>
       </c>
     </row>
-    <row r="68" spans="18:43">
+    <row r="68" spans="1:43">
+      <c r="A68">
+        <v>1902.8409999999999</v>
+      </c>
+      <c r="B68">
+        <v>3296.7440000000001</v>
+      </c>
+      <c r="C68">
+        <f t="shared" ref="C68:C70" si="7">B68-A68</f>
+        <v>1393.9030000000002</v>
+      </c>
+      <c r="D68">
+        <v>3</v>
+      </c>
+      <c r="F68" cm="1">
+        <f t="array" ref="F68:G68">LINEST(C67:C69,D67:D69^{1})</f>
+        <v>10679.576999999999</v>
+      </c>
+      <c r="G68">
+        <v>-24392.027999999998</v>
+      </c>
       <c r="R68">
         <v>36</v>
       </c>
@@ -5013,7 +6301,20 @@
         <v>-2.1457672119140599E-3</v>
       </c>
     </row>
-    <row r="69" spans="18:43">
+    <row r="69" spans="1:43">
+      <c r="A69">
+        <v>30158.742999999999</v>
+      </c>
+      <c r="B69">
+        <v>51611.423000000003</v>
+      </c>
+      <c r="C69">
+        <f t="shared" si="7"/>
+        <v>21452.680000000004</v>
+      </c>
+      <c r="D69">
+        <v>4</v>
+      </c>
       <c r="R69">
         <v>37</v>
       </c>
@@ -5064,7 +6365,20 @@
         <v>-5.2452087402343707E-3</v>
       </c>
     </row>
-    <row r="70" spans="18:43">
+    <row r="70" spans="1:43">
+      <c r="A70">
+        <v>53642.125999999997</v>
+      </c>
+      <c r="B70">
+        <v>82655.05</v>
+      </c>
+      <c r="C70">
+        <f t="shared" si="7"/>
+        <v>29012.924000000006</v>
+      </c>
+      <c r="D70">
+        <v>2</v>
+      </c>
       <c r="R70">
         <v>38</v>
       </c>
@@ -5115,7 +6429,7 @@
         <v>-5.2452087402343802E-3</v>
       </c>
     </row>
-    <row r="71" spans="18:43">
+    <row r="71" spans="1:43">
       <c r="R71">
         <v>39</v>
       </c>
@@ -5174,7 +6488,7 @@
         <v>-3.0994415283203099E-3</v>
       </c>
     </row>
-    <row r="72" spans="18:43">
+    <row r="72" spans="1:43">
       <c r="R72">
         <v>40</v>
       </c>
@@ -5237,7 +6551,7 @@
         <v>1.4305114746093702E-3</v>
       </c>
     </row>
-    <row r="73" spans="18:43">
+    <row r="73" spans="1:43">
       <c r="R73">
         <v>41</v>
       </c>
@@ -5296,7 +6610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="18:43">
+    <row r="74" spans="1:43">
       <c r="R74">
         <v>42</v>
       </c>
@@ -5351,7 +6665,7 @@
         <v>1.1920928955078201E-3</v>
       </c>
     </row>
-    <row r="75" spans="18:43">
+    <row r="75" spans="1:43">
       <c r="R75">
         <v>43</v>
       </c>
@@ -5406,7 +6720,7 @@
         <v>-1.9073486328125E-3</v>
       </c>
     </row>
-    <row r="76" spans="18:43">
+    <row r="76" spans="1:43">
       <c r="R76">
         <v>44</v>
       </c>
@@ -5461,7 +6775,7 @@
         <v>-1.096725463867184E-2</v>
       </c>
     </row>
-    <row r="77" spans="18:43">
+    <row r="77" spans="1:43">
       <c r="R77">
         <v>45</v>
       </c>
@@ -5512,7 +6826,7 @@
         <v>-6.1988830566406007E-3</v>
       </c>
     </row>
-    <row r="78" spans="18:43">
+    <row r="78" spans="1:43">
       <c r="R78">
         <v>46</v>
       </c>
@@ -5571,7 +6885,7 @@
         <v>4.2915344238281198E-3</v>
       </c>
     </row>
-    <row r="79" spans="18:43">
+    <row r="79" spans="1:43">
       <c r="V79">
         <f>AVERAGE(V33:V78)</f>
         <v>1.1247137318486744E-3</v>
@@ -5591,6 +6905,33 @@
       <c r="AQ79">
         <f>AVERAGE(AQ33:AQ78)</f>
         <v>7.7605247497558507E-3</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87">
+        <v>2</v>
+      </c>
+      <c r="B87">
+        <f>(4^A87) *(3^A87)</f>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88">
+        <v>3</v>
+      </c>
+      <c r="B88">
+        <f t="shared" ref="B88:B89" si="8">4^A88 * 3^A88</f>
+        <v>1728</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89">
+        <v>4</v>
+      </c>
+      <c r="B89">
+        <f t="shared" si="8"/>
+        <v>20736</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Check validity of approach - matrices must commute
	- valid for about 23% of operations in 2x2 circuit
	- TODO: implement op application to Laplacian for other 77% of ops
</commit_message>
<xml_diff>
--- a/charts.xlsx
+++ b/charts.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusedwards/Documents/Projects/EECE571F/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B456CA-2306-5A45-880F-C8CB823F22AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E34BD11B-8377-584C-9EBC-526B5126D58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36300" yWindow="-15240" windowWidth="31120" windowHeight="23200" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
+    <workbookView minimized="1" xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Sum after each step by default, it is faster
</commit_message>
<xml_diff>
--- a/charts.xlsx
+++ b/charts.xlsx
@@ -1,29 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusedwards/Documents/Projects/EECE571F/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E34BD11B-8377-584C-9EBC-526B5126D58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9929F4BC-8071-AB4D-A692-D77EBD09C384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
+    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v2.0" hidden="1">Sheet1!$A$66</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">Sheet1!$A$67:$A$70</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">Sheet1!$B$66</definedName>
-    <definedName name="_xlchart.v2.3" hidden="1">Sheet1!$B$67:$B$70</definedName>
-    <definedName name="_xlchart.v2.4" hidden="1">Sheet1!$C$66</definedName>
-    <definedName name="_xlchart.v2.5" hidden="1">Sheet1!$C$67:$C$70</definedName>
-  </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1399,7 +1391,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>2-Qubit Ab Initio Comparison</a:t>
+              <a:t>3-Qubit Ab Initio Comparison</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1467,7 +1459,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$D$67:$D$69</c:f>
+              <c:f>Sheet1!$D$70:$D$72</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1485,18 +1477,18 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$A$67:$A$69</c:f>
+              <c:f>Sheet1!$A$70:$A$72</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>120.083</c:v>
+                  <c:v>2.8919999999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1902.8409999999999</c:v>
+                  <c:v>3.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>30158.742999999999</c:v>
+                  <c:v>4.22</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1536,7 +1528,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$D$67:$D$69</c:f>
+              <c:f>Sheet1!$D$70:$D$72</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1554,18 +1546,18 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$67:$B$69</c:f>
+              <c:f>Sheet1!$B$70:$B$72</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>213.60900000000001</c:v>
+                  <c:v>3.0150000000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3296.7440000000001</c:v>
+                  <c:v>4.4640000000000004</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>51611.423000000003</c:v>
+                  <c:v>6.6260000000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3634,7 +3626,7 @@
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>139700</xdr:colOff>
-      <xdr:row>102</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3980,7 +3972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03013973-3BF3-2745-AF8D-DE558609215C}">
-  <dimension ref="A2:AQ89"/>
+  <dimension ref="A2:AQ90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="19" max="19" width="20.33203125" customWidth="1"/>
@@ -4159,11 +4151,11 @@
         <v>4.0531158447265599E-3</v>
       </c>
       <c r="U34" t="b">
-        <f t="shared" ref="U34:U78" si="0">T34&lt;S34</f>
+        <f t="shared" ref="U34:U79" si="0">T34&lt;S34</f>
         <v>0</v>
       </c>
       <c r="V34">
-        <f t="shared" ref="V34:V78" si="1">S34-T34</f>
+        <f t="shared" ref="V34:V79" si="1">S34-T34</f>
         <v>-9.5367431640625E-4</v>
       </c>
       <c r="X34" t="s">
@@ -4179,11 +4171,11 @@
         <v>1.5020370483398399E-2</v>
       </c>
       <c r="AE34" t="b">
-        <f t="shared" ref="AE34:AE78" si="2">AD34&lt;AC34</f>
+        <f t="shared" ref="AE34:AE79" si="2">AD34&lt;AC34</f>
         <v>0</v>
       </c>
       <c r="AF34">
-        <f t="shared" ref="AF34:AF78" si="3">AC34-AD34</f>
+        <f t="shared" ref="AF34:AF79" si="3">AC34-AD34</f>
         <v>-1.192092895507809E-2</v>
       </c>
       <c r="AJ34" t="s">
@@ -4196,15 +4188,15 @@
         <v>4.0769577026367097E-2</v>
       </c>
       <c r="AN34" t="b">
-        <f t="shared" ref="AN34:AN78" si="4">AM34&lt;AL34</f>
+        <f t="shared" ref="AN34:AN79" si="4">AM34&lt;AL34</f>
         <v>0</v>
       </c>
       <c r="AO34">
-        <f t="shared" ref="AO34:AO78" si="5">INT(AN34)</f>
+        <f t="shared" ref="AO34:AO79" si="5">INT(AN34)</f>
         <v>0</v>
       </c>
       <c r="AP34">
-        <f t="shared" ref="AP34:AP78" si="6">AL34-AM34</f>
+        <f t="shared" ref="AP34:AP79" si="6">AL34-AM34</f>
         <v>-3.6716461181640535E-2</v>
       </c>
     </row>
@@ -6150,27 +6142,27 @@
     </row>
     <row r="67" spans="1:43">
       <c r="A67">
-        <v>120.083</v>
+        <v>2.0179999999999998</v>
       </c>
       <c r="B67">
-        <v>213.60900000000001</v>
+        <v>3.9580000000000002</v>
       </c>
       <c r="C67">
         <f>B67-A67</f>
-        <v>93.52600000000001</v>
+        <v>1.9400000000000004</v>
       </c>
       <c r="D67">
         <v>2</v>
       </c>
       <c r="F67" cm="1">
         <f t="array" ref="F67:H67">LINEST(C67:C69,D67:D69^{1,2})</f>
-        <v>9379.200000000008</v>
+        <v>4.1025000000000009</v>
       </c>
       <c r="G67">
-        <v>-45595.623000000043</v>
+        <v>-22.966500000000007</v>
       </c>
       <c r="H67">
-        <v>53767.972000000053</v>
+        <v>31.463000000000015</v>
       </c>
       <c r="R67">
         <v>35</v>
@@ -6232,24 +6224,24 @@
     </row>
     <row r="68" spans="1:43">
       <c r="A68">
-        <v>1902.8409999999999</v>
+        <v>3.4209999999999998</v>
       </c>
       <c r="B68">
-        <v>3296.7440000000001</v>
+        <v>2.907</v>
       </c>
       <c r="C68">
-        <f t="shared" ref="C68:C70" si="7">B68-A68</f>
-        <v>1393.9030000000002</v>
+        <f t="shared" ref="C68:C76" si="7">B68-A68</f>
+        <v>-0.51399999999999979</v>
       </c>
       <c r="D68">
         <v>3</v>
       </c>
       <c r="F68" cm="1">
         <f t="array" ref="F68:G68">LINEST(C67:C69,D67:D69^{1})</f>
-        <v>10679.576999999999</v>
+        <v>1.6484999999999999</v>
       </c>
       <c r="G68">
-        <v>-24392.027999999998</v>
+        <v>-2.724499999999999</v>
       </c>
       <c r="R68">
         <v>36</v>
@@ -6303,14 +6295,14 @@
     </row>
     <row r="69" spans="1:43">
       <c r="A69">
-        <v>30158.742999999999</v>
+        <v>2.0539999999999998</v>
       </c>
       <c r="B69">
-        <v>51611.423000000003</v>
+        <v>7.2910000000000004</v>
       </c>
       <c r="C69">
         <f t="shared" si="7"/>
-        <v>21452.680000000004</v>
+        <v>5.2370000000000001</v>
       </c>
       <c r="D69">
         <v>4</v>
@@ -6367,14 +6359,14 @@
     </row>
     <row r="70" spans="1:43">
       <c r="A70">
-        <v>53642.125999999997</v>
+        <v>2.8919999999999999</v>
       </c>
       <c r="B70">
-        <v>82655.05</v>
+        <v>3.0150000000000001</v>
       </c>
       <c r="C70">
         <f t="shared" si="7"/>
-        <v>29012.924000000006</v>
+        <v>0.12300000000000022</v>
       </c>
       <c r="D70">
         <v>2</v>
@@ -6430,6 +6422,19 @@
       </c>
     </row>
     <row r="71" spans="1:43">
+      <c r="A71">
+        <v>3.75</v>
+      </c>
+      <c r="B71">
+        <v>4.4640000000000004</v>
+      </c>
+      <c r="C71">
+        <f t="shared" si="7"/>
+        <v>0.71400000000000041</v>
+      </c>
+      <c r="D71">
+        <v>3</v>
+      </c>
       <c r="R71">
         <v>39</v>
       </c>
@@ -6489,6 +6494,19 @@
       </c>
     </row>
     <row r="72" spans="1:43">
+      <c r="A72">
+        <v>4.22</v>
+      </c>
+      <c r="B72">
+        <v>6.6260000000000003</v>
+      </c>
+      <c r="C72">
+        <f t="shared" si="7"/>
+        <v>2.4060000000000006</v>
+      </c>
+      <c r="D72">
+        <v>4</v>
+      </c>
       <c r="R72">
         <v>40</v>
       </c>
@@ -6552,143 +6570,131 @@
       </c>
     </row>
     <row r="73" spans="1:43">
-      <c r="R73">
+      <c r="A73">
+        <v>7.7039999999999997</v>
+      </c>
+      <c r="B73">
+        <v>9.2200000000000006</v>
+      </c>
+      <c r="C73">
+        <f t="shared" si="7"/>
+        <v>1.5160000000000009</v>
+      </c>
+      <c r="D73">
+        <v>5</v>
+      </c>
+      <c r="S73" s="1"/>
+      <c r="T73" s="1"/>
+      <c r="AC73" s="1"/>
+      <c r="AD73" s="1"/>
+      <c r="AL73" s="1"/>
+      <c r="AM73" s="1"/>
+    </row>
+    <row r="74" spans="1:43">
+      <c r="A74">
+        <v>2.488</v>
+      </c>
+      <c r="B74">
+        <v>4.923</v>
+      </c>
+      <c r="C74">
+        <f t="shared" si="7"/>
+        <v>2.4350000000000001</v>
+      </c>
+      <c r="D74">
+        <v>2</v>
+      </c>
+      <c r="R74">
         <v>41</v>
       </c>
-      <c r="S73" s="1">
+      <c r="S74" s="1">
         <v>2.1457672119140599E-3</v>
       </c>
-      <c r="T73" s="1">
+      <c r="T74" s="1">
         <v>9.5367431640625E-4</v>
       </c>
-      <c r="U73" t="b">
+      <c r="U74" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="V73">
+      <c r="V74">
         <f t="shared" si="1"/>
         <v>1.1920928955078099E-3</v>
       </c>
-      <c r="W73" cm="1">
-        <f t="array" ref="W73">IF(U73, V73, null)</f>
+      <c r="W74" cm="1">
+        <f t="array" ref="W74">IF(U74, V74, null)</f>
         <v>1.1920928955078099E-3</v>
       </c>
-      <c r="AC73" s="1">
+      <c r="AC74" s="1">
         <v>3.0994415283203099E-3</v>
       </c>
-      <c r="AD73" s="1">
+      <c r="AD74" s="1">
         <v>1.9073486328125E-3</v>
       </c>
-      <c r="AE73" t="b">
+      <c r="AE74" t="b">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AF73">
+      <c r="AF74">
         <f t="shared" si="3"/>
         <v>1.1920928955078099E-3</v>
       </c>
-      <c r="AG73" cm="1">
-        <f t="array" ref="AG73">IF(AE73,AF73,null)</f>
+      <c r="AG74" cm="1">
+        <f t="array" ref="AG74">IF(AE74,AF74,null)</f>
         <v>1.1920928955078099E-3</v>
       </c>
-      <c r="AL73" s="1">
+      <c r="AL74" s="1">
         <v>2.1457672119140599E-3</v>
       </c>
-      <c r="AM73" s="1">
+      <c r="AM74" s="1">
         <v>2.1457672119140599E-3</v>
-      </c>
-      <c r="AN73" t="b">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AO73">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="AP73">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:43">
-      <c r="R74">
-        <v>42</v>
-      </c>
-      <c r="S74" s="1">
-        <v>1.9073486328125E-3</v>
-      </c>
-      <c r="T74" s="1">
-        <v>1.9073486328125E-3</v>
-      </c>
-      <c r="U74" t="b">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="V74">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AC74" s="1">
-        <v>2.1457672119140599E-3</v>
-      </c>
-      <c r="AD74" s="1">
-        <v>2.1457672119140599E-3</v>
-      </c>
-      <c r="AE74" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF74">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AL74" s="1">
-        <v>2.86102294921875E-3</v>
-      </c>
-      <c r="AM74" s="1">
-        <v>1.6689300537109299E-3</v>
       </c>
       <c r="AN74" t="b">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO74">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP74">
         <f t="shared" si="6"/>
-        <v>1.1920928955078201E-3</v>
-      </c>
-      <c r="AQ74" cm="1">
-        <f t="array" ref="AQ74">IF(AN74,AP74,null)</f>
-        <v>1.1920928955078201E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:43">
+      <c r="A75">
+        <v>6.9729999999999999</v>
+      </c>
+      <c r="B75">
+        <v>9.2539999999999996</v>
+      </c>
+      <c r="C75">
+        <f t="shared" si="7"/>
+        <v>2.2809999999999997</v>
+      </c>
+      <c r="D75">
+        <v>3</v>
+      </c>
       <c r="R75">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S75" s="1">
-        <v>3.0994415283203099E-3</v>
+        <v>1.9073486328125E-3</v>
       </c>
       <c r="T75" s="1">
         <v>1.9073486328125E-3</v>
       </c>
       <c r="U75" t="b">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V75">
         <f t="shared" si="1"/>
-        <v>1.1920928955078099E-3</v>
-      </c>
-      <c r="W75" cm="1">
-        <f t="array" ref="W75">IF(U75, V75, null)</f>
-        <v>1.1920928955078099E-3</v>
+        <v>0</v>
       </c>
       <c r="AC75" s="1">
-        <v>1.9073486328125E-3</v>
+        <v>2.1457672119140599E-3</v>
       </c>
       <c r="AD75" s="1">
         <v>2.1457672119140599E-3</v>
@@ -6699,33 +6705,50 @@
       </c>
       <c r="AF75">
         <f t="shared" si="3"/>
-        <v>-2.384185791015599E-4</v>
+        <v>0</v>
       </c>
       <c r="AL75" s="1">
-        <v>3.0994415283203099E-3</v>
+        <v>2.86102294921875E-3</v>
       </c>
       <c r="AM75" s="1">
-        <v>5.0067901611328099E-3</v>
+        <v>1.6689300537109299E-3</v>
       </c>
       <c r="AN75" t="b">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO75">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP75">
         <f t="shared" si="6"/>
-        <v>-1.9073486328125E-3</v>
+        <v>1.1920928955078201E-3</v>
+      </c>
+      <c r="AQ75" cm="1">
+        <f t="array" ref="AQ75">IF(AN75,AP75,null)</f>
+        <v>1.1920928955078201E-3</v>
       </c>
     </row>
     <row r="76" spans="1:43">
+      <c r="A76">
+        <v>7.9989999999999997</v>
+      </c>
+      <c r="B76">
+        <v>9.0169999999999995</v>
+      </c>
+      <c r="C76">
+        <f t="shared" si="7"/>
+        <v>1.0179999999999998</v>
+      </c>
+      <c r="D76">
+        <v>4</v>
+      </c>
       <c r="R76">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S76" s="1">
-        <v>2.1457672119140599E-3</v>
+        <v>3.0994415283203099E-3</v>
       </c>
       <c r="T76" s="1">
         <v>1.9073486328125E-3</v>
@@ -6736,17 +6759,17 @@
       </c>
       <c r="V76">
         <f t="shared" si="1"/>
-        <v>2.384185791015599E-4</v>
+        <v>1.1920928955078099E-3</v>
       </c>
       <c r="W76" cm="1">
         <f t="array" ref="W76">IF(U76, V76, null)</f>
-        <v>2.384185791015599E-4</v>
+        <v>1.1920928955078099E-3</v>
       </c>
       <c r="AC76" s="1">
         <v>1.9073486328125E-3</v>
       </c>
       <c r="AD76" s="1">
-        <v>6.9141387939453099E-3</v>
+        <v>2.1457672119140599E-3</v>
       </c>
       <c r="AE76" t="b">
         <f t="shared" si="2"/>
@@ -6754,13 +6777,13 @@
       </c>
       <c r="AF76">
         <f t="shared" si="3"/>
-        <v>-5.0067901611328099E-3</v>
+        <v>-2.384185791015599E-4</v>
       </c>
       <c r="AL76" s="1">
-        <v>2.1457672119140599E-3</v>
+        <v>3.0994415283203099E-3</v>
       </c>
       <c r="AM76" s="1">
-        <v>1.3113021850585899E-2</v>
+        <v>5.0067901611328099E-3</v>
       </c>
       <c r="AN76" t="b">
         <f t="shared" si="4"/>
@@ -6772,32 +6795,36 @@
       </c>
       <c r="AP76">
         <f t="shared" si="6"/>
-        <v>-1.096725463867184E-2</v>
+        <v>-1.9073486328125E-3</v>
       </c>
     </row>
     <row r="77" spans="1:43">
       <c r="R77">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S77" s="1">
-        <v>2.86102294921875E-3</v>
+        <v>2.1457672119140599E-3</v>
       </c>
       <c r="T77" s="1">
-        <v>4.2915344238281198E-3</v>
+        <v>1.9073486328125E-3</v>
       </c>
       <c r="U77" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V77">
         <f t="shared" si="1"/>
-        <v>-1.4305114746093698E-3</v>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="W77" cm="1">
+        <f t="array" ref="W77">IF(U77, V77, null)</f>
+        <v>2.384185791015599E-4</v>
       </c>
       <c r="AC77" s="1">
-        <v>3.0994415283203099E-3</v>
+        <v>1.9073486328125E-3</v>
       </c>
       <c r="AD77" s="1">
-        <v>6.1988830566406198E-3</v>
+        <v>6.9141387939453099E-3</v>
       </c>
       <c r="AE77" t="b">
         <f t="shared" si="2"/>
@@ -6805,13 +6832,13 @@
       </c>
       <c r="AF77">
         <f t="shared" si="3"/>
-        <v>-3.0994415283203099E-3</v>
+        <v>-5.0067901611328099E-3</v>
       </c>
       <c r="AL77" s="1">
-        <v>3.814697265625E-3</v>
+        <v>2.1457672119140599E-3</v>
       </c>
       <c r="AM77" s="1">
-        <v>1.0013580322265601E-2</v>
+        <v>1.3113021850585899E-2</v>
       </c>
       <c r="AN77" t="b">
         <f t="shared" si="4"/>
@@ -6823,36 +6850,32 @@
       </c>
       <c r="AP77">
         <f t="shared" si="6"/>
-        <v>-6.1988830566406007E-3</v>
+        <v>-1.096725463867184E-2</v>
       </c>
     </row>
     <row r="78" spans="1:43">
       <c r="R78">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S78" s="1">
-        <v>1.9073486328125E-3</v>
+        <v>2.86102294921875E-3</v>
       </c>
       <c r="T78" s="1">
-        <v>9.5367431640625E-4</v>
+        <v>4.2915344238281198E-3</v>
       </c>
       <c r="U78" t="b">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V78">
         <f t="shared" si="1"/>
-        <v>9.5367431640625E-4</v>
-      </c>
-      <c r="W78" cm="1">
-        <f t="array" ref="W78">IF(U78, V78, null)</f>
-        <v>9.5367431640625E-4</v>
+        <v>-1.4305114746093698E-3</v>
       </c>
       <c r="AC78" s="1">
-        <v>1.9073486328125E-3</v>
+        <v>3.0994415283203099E-3</v>
       </c>
       <c r="AD78" s="1">
-        <v>2.1457672119140599E-3</v>
+        <v>6.1988830566406198E-3</v>
       </c>
       <c r="AE78" t="b">
         <f t="shared" si="2"/>
@@ -6860,76 +6883,131 @@
       </c>
       <c r="AF78">
         <f t="shared" si="3"/>
-        <v>-2.384185791015599E-4</v>
+        <v>-3.0994415283203099E-3</v>
       </c>
       <c r="AL78" s="1">
-        <v>6.1988830566406198E-3</v>
+        <v>3.814697265625E-3</v>
       </c>
       <c r="AM78" s="1">
-        <v>1.9073486328125E-3</v>
+        <v>1.0013580322265601E-2</v>
       </c>
       <c r="AN78" t="b">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO78">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP78">
         <f t="shared" si="6"/>
-        <v>4.2915344238281198E-3</v>
-      </c>
-      <c r="AQ78" cm="1">
-        <f t="array" ref="AQ78">IF(AN78,AP78,null)</f>
-        <v>4.2915344238281198E-3</v>
+        <v>-6.1988830566406007E-3</v>
       </c>
     </row>
     <row r="79" spans="1:43">
+      <c r="R79">
+        <v>46</v>
+      </c>
+      <c r="S79" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T79" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U79" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
       <c r="V79">
-        <f>AVERAGE(V33:V78)</f>
+        <f t="shared" si="1"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="W79" cm="1">
+        <f t="array" ref="W79">IF(U79, V79, null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AC79" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD79" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE79" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF79">
+        <f t="shared" si="3"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AL79" s="1">
+        <v>6.1988830566406198E-3</v>
+      </c>
+      <c r="AM79" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AN79" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO79">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP79">
+        <f t="shared" si="6"/>
+        <v>4.2915344238281198E-3</v>
+      </c>
+      <c r="AQ79" cm="1">
+        <f t="array" ref="AQ79">IF(AN79,AP79,null)</f>
+        <v>4.2915344238281198E-3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:43">
+      <c r="V80">
+        <f>AVERAGE(V33:V79)</f>
         <v>1.1247137318486744E-3</v>
       </c>
-      <c r="W79">
-        <f>AVERAGE(W33:W78)</f>
+      <c r="W80">
+        <f>AVERAGE(W33:W79)</f>
         <v>1.7657876014709455E-3</v>
       </c>
-      <c r="AG79">
-        <f>AVERAGE(AG33:AG75)</f>
+      <c r="AG80">
+        <f>AVERAGE(AG33:AG76)</f>
         <v>3.5674483687789305E-3</v>
       </c>
-      <c r="AO79">
-        <f>SUM(AO33:AO78)</f>
+      <c r="AO80">
+        <f>SUM(AO33:AO79)</f>
         <v>20</v>
       </c>
-      <c r="AQ79">
-        <f>AVERAGE(AQ33:AQ78)</f>
+      <c r="AQ80">
+        <f>AVERAGE(AQ33:AQ79)</f>
         <v>7.7605247497558507E-3</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2">
-      <c r="A87">
-        <v>2</v>
-      </c>
-      <c r="B87">
-        <f>(4^A87) *(3^A87)</f>
-        <v>144</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B88">
-        <f t="shared" ref="B88:B89" si="8">4^A88 * 3^A88</f>
-        <v>1728</v>
+        <f>(4^A88) *(3^A88)</f>
+        <v>144</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89">
+        <v>3</v>
+      </c>
+      <c r="B89">
+        <f t="shared" ref="B89:B90" si="8">4^A89 * 3^A89</f>
+        <v>1728</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90">
         <v>4</v>
       </c>
-      <c r="B89">
+      <c r="B90">
         <f t="shared" si="8"/>
         <v>20736</v>
       </c>

</xml_diff>

<commit_message>
Remove and untrack data from git lfs
</commit_message>
<xml_diff>
--- a/charts.xlsx
+++ b/charts.xlsx
@@ -1,29 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marcusedwards/Documents/Projects/EECE571F/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E34BD11B-8377-584C-9EBC-526B5126D58F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9929F4BC-8071-AB4D-A692-D77EBD09C384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
+    <workbookView xWindow="1100" yWindow="820" windowWidth="28040" windowHeight="17440" xr2:uid="{B5BBAECF-680A-EA45-B7E1-873697CAF963}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v2.0" hidden="1">Sheet1!$A$66</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">Sheet1!$A$67:$A$70</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">Sheet1!$B$66</definedName>
-    <definedName name="_xlchart.v2.3" hidden="1">Sheet1!$B$67:$B$70</definedName>
-    <definedName name="_xlchart.v2.4" hidden="1">Sheet1!$C$66</definedName>
-    <definedName name="_xlchart.v2.5" hidden="1">Sheet1!$C$67:$C$70</definedName>
-  </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1399,7 +1391,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>2-Qubit Ab Initio Comparison</a:t>
+              <a:t>3-Qubit Ab Initio Comparison</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1467,7 +1459,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$D$67:$D$69</c:f>
+              <c:f>Sheet1!$D$70:$D$72</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1485,18 +1477,18 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$A$67:$A$69</c:f>
+              <c:f>Sheet1!$A$70:$A$72</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>120.083</c:v>
+                  <c:v>2.8919999999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1902.8409999999999</c:v>
+                  <c:v>3.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>30158.742999999999</c:v>
+                  <c:v>4.22</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1536,7 +1528,7 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$D$67:$D$69</c:f>
+              <c:f>Sheet1!$D$70:$D$72</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
@@ -1554,18 +1546,18 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$67:$B$69</c:f>
+              <c:f>Sheet1!$B$70:$B$72</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>213.60900000000001</c:v>
+                  <c:v>3.0150000000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3296.7440000000001</c:v>
+                  <c:v>4.4640000000000004</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>51611.423000000003</c:v>
+                  <c:v>6.6260000000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3634,7 +3626,7 @@
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>139700</xdr:colOff>
-      <xdr:row>102</xdr:row>
+      <xdr:row>103</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3980,7 +3972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03013973-3BF3-2745-AF8D-DE558609215C}">
-  <dimension ref="A2:AQ89"/>
+  <dimension ref="A2:AQ90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="19" max="19" width="20.33203125" customWidth="1"/>
@@ -4159,11 +4151,11 @@
         <v>4.0531158447265599E-3</v>
       </c>
       <c r="U34" t="b">
-        <f t="shared" ref="U34:U78" si="0">T34&lt;S34</f>
+        <f t="shared" ref="U34:U79" si="0">T34&lt;S34</f>
         <v>0</v>
       </c>
       <c r="V34">
-        <f t="shared" ref="V34:V78" si="1">S34-T34</f>
+        <f t="shared" ref="V34:V79" si="1">S34-T34</f>
         <v>-9.5367431640625E-4</v>
       </c>
       <c r="X34" t="s">
@@ -4179,11 +4171,11 @@
         <v>1.5020370483398399E-2</v>
       </c>
       <c r="AE34" t="b">
-        <f t="shared" ref="AE34:AE78" si="2">AD34&lt;AC34</f>
+        <f t="shared" ref="AE34:AE79" si="2">AD34&lt;AC34</f>
         <v>0</v>
       </c>
       <c r="AF34">
-        <f t="shared" ref="AF34:AF78" si="3">AC34-AD34</f>
+        <f t="shared" ref="AF34:AF79" si="3">AC34-AD34</f>
         <v>-1.192092895507809E-2</v>
       </c>
       <c r="AJ34" t="s">
@@ -4196,15 +4188,15 @@
         <v>4.0769577026367097E-2</v>
       </c>
       <c r="AN34" t="b">
-        <f t="shared" ref="AN34:AN78" si="4">AM34&lt;AL34</f>
+        <f t="shared" ref="AN34:AN79" si="4">AM34&lt;AL34</f>
         <v>0</v>
       </c>
       <c r="AO34">
-        <f t="shared" ref="AO34:AO78" si="5">INT(AN34)</f>
+        <f t="shared" ref="AO34:AO79" si="5">INT(AN34)</f>
         <v>0</v>
       </c>
       <c r="AP34">
-        <f t="shared" ref="AP34:AP78" si="6">AL34-AM34</f>
+        <f t="shared" ref="AP34:AP79" si="6">AL34-AM34</f>
         <v>-3.6716461181640535E-2</v>
       </c>
     </row>
@@ -6150,27 +6142,27 @@
     </row>
     <row r="67" spans="1:43">
       <c r="A67">
-        <v>120.083</v>
+        <v>2.0179999999999998</v>
       </c>
       <c r="B67">
-        <v>213.60900000000001</v>
+        <v>3.9580000000000002</v>
       </c>
       <c r="C67">
         <f>B67-A67</f>
-        <v>93.52600000000001</v>
+        <v>1.9400000000000004</v>
       </c>
       <c r="D67">
         <v>2</v>
       </c>
       <c r="F67" cm="1">
         <f t="array" ref="F67:H67">LINEST(C67:C69,D67:D69^{1,2})</f>
-        <v>9379.200000000008</v>
+        <v>4.1025000000000009</v>
       </c>
       <c r="G67">
-        <v>-45595.623000000043</v>
+        <v>-22.966500000000007</v>
       </c>
       <c r="H67">
-        <v>53767.972000000053</v>
+        <v>31.463000000000015</v>
       </c>
       <c r="R67">
         <v>35</v>
@@ -6232,24 +6224,24 @@
     </row>
     <row r="68" spans="1:43">
       <c r="A68">
-        <v>1902.8409999999999</v>
+        <v>3.4209999999999998</v>
       </c>
       <c r="B68">
-        <v>3296.7440000000001</v>
+        <v>2.907</v>
       </c>
       <c r="C68">
-        <f t="shared" ref="C68:C70" si="7">B68-A68</f>
-        <v>1393.9030000000002</v>
+        <f t="shared" ref="C68:C76" si="7">B68-A68</f>
+        <v>-0.51399999999999979</v>
       </c>
       <c r="D68">
         <v>3</v>
       </c>
       <c r="F68" cm="1">
         <f t="array" ref="F68:G68">LINEST(C67:C69,D67:D69^{1})</f>
-        <v>10679.576999999999</v>
+        <v>1.6484999999999999</v>
       </c>
       <c r="G68">
-        <v>-24392.027999999998</v>
+        <v>-2.724499999999999</v>
       </c>
       <c r="R68">
         <v>36</v>
@@ -6303,14 +6295,14 @@
     </row>
     <row r="69" spans="1:43">
       <c r="A69">
-        <v>30158.742999999999</v>
+        <v>2.0539999999999998</v>
       </c>
       <c r="B69">
-        <v>51611.423000000003</v>
+        <v>7.2910000000000004</v>
       </c>
       <c r="C69">
         <f t="shared" si="7"/>
-        <v>21452.680000000004</v>
+        <v>5.2370000000000001</v>
       </c>
       <c r="D69">
         <v>4</v>
@@ -6367,14 +6359,14 @@
     </row>
     <row r="70" spans="1:43">
       <c r="A70">
-        <v>53642.125999999997</v>
+        <v>2.8919999999999999</v>
       </c>
       <c r="B70">
-        <v>82655.05</v>
+        <v>3.0150000000000001</v>
       </c>
       <c r="C70">
         <f t="shared" si="7"/>
-        <v>29012.924000000006</v>
+        <v>0.12300000000000022</v>
       </c>
       <c r="D70">
         <v>2</v>
@@ -6430,6 +6422,19 @@
       </c>
     </row>
     <row r="71" spans="1:43">
+      <c r="A71">
+        <v>3.75</v>
+      </c>
+      <c r="B71">
+        <v>4.4640000000000004</v>
+      </c>
+      <c r="C71">
+        <f t="shared" si="7"/>
+        <v>0.71400000000000041</v>
+      </c>
+      <c r="D71">
+        <v>3</v>
+      </c>
       <c r="R71">
         <v>39</v>
       </c>
@@ -6489,6 +6494,19 @@
       </c>
     </row>
     <row r="72" spans="1:43">
+      <c r="A72">
+        <v>4.22</v>
+      </c>
+      <c r="B72">
+        <v>6.6260000000000003</v>
+      </c>
+      <c r="C72">
+        <f t="shared" si="7"/>
+        <v>2.4060000000000006</v>
+      </c>
+      <c r="D72">
+        <v>4</v>
+      </c>
       <c r="R72">
         <v>40</v>
       </c>
@@ -6552,143 +6570,131 @@
       </c>
     </row>
     <row r="73" spans="1:43">
-      <c r="R73">
+      <c r="A73">
+        <v>7.7039999999999997</v>
+      </c>
+      <c r="B73">
+        <v>9.2200000000000006</v>
+      </c>
+      <c r="C73">
+        <f t="shared" si="7"/>
+        <v>1.5160000000000009</v>
+      </c>
+      <c r="D73">
+        <v>5</v>
+      </c>
+      <c r="S73" s="1"/>
+      <c r="T73" s="1"/>
+      <c r="AC73" s="1"/>
+      <c r="AD73" s="1"/>
+      <c r="AL73" s="1"/>
+      <c r="AM73" s="1"/>
+    </row>
+    <row r="74" spans="1:43">
+      <c r="A74">
+        <v>2.488</v>
+      </c>
+      <c r="B74">
+        <v>4.923</v>
+      </c>
+      <c r="C74">
+        <f t="shared" si="7"/>
+        <v>2.4350000000000001</v>
+      </c>
+      <c r="D74">
+        <v>2</v>
+      </c>
+      <c r="R74">
         <v>41</v>
       </c>
-      <c r="S73" s="1">
+      <c r="S74" s="1">
         <v>2.1457672119140599E-3</v>
       </c>
-      <c r="T73" s="1">
+      <c r="T74" s="1">
         <v>9.5367431640625E-4</v>
       </c>
-      <c r="U73" t="b">
+      <c r="U74" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="V73">
+      <c r="V74">
         <f t="shared" si="1"/>
         <v>1.1920928955078099E-3</v>
       </c>
-      <c r="W73" cm="1">
-        <f t="array" ref="W73">IF(U73, V73, null)</f>
+      <c r="W74" cm="1">
+        <f t="array" ref="W74">IF(U74, V74, null)</f>
         <v>1.1920928955078099E-3</v>
       </c>
-      <c r="AC73" s="1">
+      <c r="AC74" s="1">
         <v>3.0994415283203099E-3</v>
       </c>
-      <c r="AD73" s="1">
+      <c r="AD74" s="1">
         <v>1.9073486328125E-3</v>
       </c>
-      <c r="AE73" t="b">
+      <c r="AE74" t="b">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="AF73">
+      <c r="AF74">
         <f t="shared" si="3"/>
         <v>1.1920928955078099E-3</v>
       </c>
-      <c r="AG73" cm="1">
-        <f t="array" ref="AG73">IF(AE73,AF73,null)</f>
+      <c r="AG74" cm="1">
+        <f t="array" ref="AG74">IF(AE74,AF74,null)</f>
         <v>1.1920928955078099E-3</v>
       </c>
-      <c r="AL73" s="1">
+      <c r="AL74" s="1">
         <v>2.1457672119140599E-3</v>
       </c>
-      <c r="AM73" s="1">
+      <c r="AM74" s="1">
         <v>2.1457672119140599E-3</v>
-      </c>
-      <c r="AN73" t="b">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="AO73">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="AP73">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:43">
-      <c r="R74">
-        <v>42</v>
-      </c>
-      <c r="S74" s="1">
-        <v>1.9073486328125E-3</v>
-      </c>
-      <c r="T74" s="1">
-        <v>1.9073486328125E-3</v>
-      </c>
-      <c r="U74" t="b">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="V74">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="AC74" s="1">
-        <v>2.1457672119140599E-3</v>
-      </c>
-      <c r="AD74" s="1">
-        <v>2.1457672119140599E-3</v>
-      </c>
-      <c r="AE74" t="b">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="AF74">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="AL74" s="1">
-        <v>2.86102294921875E-3</v>
-      </c>
-      <c r="AM74" s="1">
-        <v>1.6689300537109299E-3</v>
       </c>
       <c r="AN74" t="b">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO74">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP74">
         <f t="shared" si="6"/>
-        <v>1.1920928955078201E-3</v>
-      </c>
-      <c r="AQ74" cm="1">
-        <f t="array" ref="AQ74">IF(AN74,AP74,null)</f>
-        <v>1.1920928955078201E-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75" spans="1:43">
+      <c r="A75">
+        <v>6.9729999999999999</v>
+      </c>
+      <c r="B75">
+        <v>9.2539999999999996</v>
+      </c>
+      <c r="C75">
+        <f t="shared" si="7"/>
+        <v>2.2809999999999997</v>
+      </c>
+      <c r="D75">
+        <v>3</v>
+      </c>
       <c r="R75">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="S75" s="1">
-        <v>3.0994415283203099E-3</v>
+        <v>1.9073486328125E-3</v>
       </c>
       <c r="T75" s="1">
         <v>1.9073486328125E-3</v>
       </c>
       <c r="U75" t="b">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V75">
         <f t="shared" si="1"/>
-        <v>1.1920928955078099E-3</v>
-      </c>
-      <c r="W75" cm="1">
-        <f t="array" ref="W75">IF(U75, V75, null)</f>
-        <v>1.1920928955078099E-3</v>
+        <v>0</v>
       </c>
       <c r="AC75" s="1">
-        <v>1.9073486328125E-3</v>
+        <v>2.1457672119140599E-3</v>
       </c>
       <c r="AD75" s="1">
         <v>2.1457672119140599E-3</v>
@@ -6699,33 +6705,50 @@
       </c>
       <c r="AF75">
         <f t="shared" si="3"/>
-        <v>-2.384185791015599E-4</v>
+        <v>0</v>
       </c>
       <c r="AL75" s="1">
-        <v>3.0994415283203099E-3</v>
+        <v>2.86102294921875E-3</v>
       </c>
       <c r="AM75" s="1">
-        <v>5.0067901611328099E-3</v>
+        <v>1.6689300537109299E-3</v>
       </c>
       <c r="AN75" t="b">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO75">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP75">
         <f t="shared" si="6"/>
-        <v>-1.9073486328125E-3</v>
+        <v>1.1920928955078201E-3</v>
+      </c>
+      <c r="AQ75" cm="1">
+        <f t="array" ref="AQ75">IF(AN75,AP75,null)</f>
+        <v>1.1920928955078201E-3</v>
       </c>
     </row>
     <row r="76" spans="1:43">
+      <c r="A76">
+        <v>7.9989999999999997</v>
+      </c>
+      <c r="B76">
+        <v>9.0169999999999995</v>
+      </c>
+      <c r="C76">
+        <f t="shared" si="7"/>
+        <v>1.0179999999999998</v>
+      </c>
+      <c r="D76">
+        <v>4</v>
+      </c>
       <c r="R76">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S76" s="1">
-        <v>2.1457672119140599E-3</v>
+        <v>3.0994415283203099E-3</v>
       </c>
       <c r="T76" s="1">
         <v>1.9073486328125E-3</v>
@@ -6736,17 +6759,17 @@
       </c>
       <c r="V76">
         <f t="shared" si="1"/>
-        <v>2.384185791015599E-4</v>
+        <v>1.1920928955078099E-3</v>
       </c>
       <c r="W76" cm="1">
         <f t="array" ref="W76">IF(U76, V76, null)</f>
-        <v>2.384185791015599E-4</v>
+        <v>1.1920928955078099E-3</v>
       </c>
       <c r="AC76" s="1">
         <v>1.9073486328125E-3</v>
       </c>
       <c r="AD76" s="1">
-        <v>6.9141387939453099E-3</v>
+        <v>2.1457672119140599E-3</v>
       </c>
       <c r="AE76" t="b">
         <f t="shared" si="2"/>
@@ -6754,13 +6777,13 @@
       </c>
       <c r="AF76">
         <f t="shared" si="3"/>
-        <v>-5.0067901611328099E-3</v>
+        <v>-2.384185791015599E-4</v>
       </c>
       <c r="AL76" s="1">
-        <v>2.1457672119140599E-3</v>
+        <v>3.0994415283203099E-3</v>
       </c>
       <c r="AM76" s="1">
-        <v>1.3113021850585899E-2</v>
+        <v>5.0067901611328099E-3</v>
       </c>
       <c r="AN76" t="b">
         <f t="shared" si="4"/>
@@ -6772,32 +6795,36 @@
       </c>
       <c r="AP76">
         <f t="shared" si="6"/>
-        <v>-1.096725463867184E-2</v>
+        <v>-1.9073486328125E-3</v>
       </c>
     </row>
     <row r="77" spans="1:43">
       <c r="R77">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S77" s="1">
-        <v>2.86102294921875E-3</v>
+        <v>2.1457672119140599E-3</v>
       </c>
       <c r="T77" s="1">
-        <v>4.2915344238281198E-3</v>
+        <v>1.9073486328125E-3</v>
       </c>
       <c r="U77" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V77">
         <f t="shared" si="1"/>
-        <v>-1.4305114746093698E-3</v>
+        <v>2.384185791015599E-4</v>
+      </c>
+      <c r="W77" cm="1">
+        <f t="array" ref="W77">IF(U77, V77, null)</f>
+        <v>2.384185791015599E-4</v>
       </c>
       <c r="AC77" s="1">
-        <v>3.0994415283203099E-3</v>
+        <v>1.9073486328125E-3</v>
       </c>
       <c r="AD77" s="1">
-        <v>6.1988830566406198E-3</v>
+        <v>6.9141387939453099E-3</v>
       </c>
       <c r="AE77" t="b">
         <f t="shared" si="2"/>
@@ -6805,13 +6832,13 @@
       </c>
       <c r="AF77">
         <f t="shared" si="3"/>
-        <v>-3.0994415283203099E-3</v>
+        <v>-5.0067901611328099E-3</v>
       </c>
       <c r="AL77" s="1">
-        <v>3.814697265625E-3</v>
+        <v>2.1457672119140599E-3</v>
       </c>
       <c r="AM77" s="1">
-        <v>1.0013580322265601E-2</v>
+        <v>1.3113021850585899E-2</v>
       </c>
       <c r="AN77" t="b">
         <f t="shared" si="4"/>
@@ -6823,36 +6850,32 @@
       </c>
       <c r="AP77">
         <f t="shared" si="6"/>
-        <v>-6.1988830566406007E-3</v>
+        <v>-1.096725463867184E-2</v>
       </c>
     </row>
     <row r="78" spans="1:43">
       <c r="R78">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S78" s="1">
-        <v>1.9073486328125E-3</v>
+        <v>2.86102294921875E-3</v>
       </c>
       <c r="T78" s="1">
-        <v>9.5367431640625E-4</v>
+        <v>4.2915344238281198E-3</v>
       </c>
       <c r="U78" t="b">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V78">
         <f t="shared" si="1"/>
-        <v>9.5367431640625E-4</v>
-      </c>
-      <c r="W78" cm="1">
-        <f t="array" ref="W78">IF(U78, V78, null)</f>
-        <v>9.5367431640625E-4</v>
+        <v>-1.4305114746093698E-3</v>
       </c>
       <c r="AC78" s="1">
-        <v>1.9073486328125E-3</v>
+        <v>3.0994415283203099E-3</v>
       </c>
       <c r="AD78" s="1">
-        <v>2.1457672119140599E-3</v>
+        <v>6.1988830566406198E-3</v>
       </c>
       <c r="AE78" t="b">
         <f t="shared" si="2"/>
@@ -6860,76 +6883,131 @@
       </c>
       <c r="AF78">
         <f t="shared" si="3"/>
-        <v>-2.384185791015599E-4</v>
+        <v>-3.0994415283203099E-3</v>
       </c>
       <c r="AL78" s="1">
-        <v>6.1988830566406198E-3</v>
+        <v>3.814697265625E-3</v>
       </c>
       <c r="AM78" s="1">
-        <v>1.9073486328125E-3</v>
+        <v>1.0013580322265601E-2</v>
       </c>
       <c r="AN78" t="b">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO78">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP78">
         <f t="shared" si="6"/>
-        <v>4.2915344238281198E-3</v>
-      </c>
-      <c r="AQ78" cm="1">
-        <f t="array" ref="AQ78">IF(AN78,AP78,null)</f>
-        <v>4.2915344238281198E-3</v>
+        <v>-6.1988830566406007E-3</v>
       </c>
     </row>
     <row r="79" spans="1:43">
+      <c r="R79">
+        <v>46</v>
+      </c>
+      <c r="S79" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="T79" s="1">
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="U79" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
       <c r="V79">
-        <f>AVERAGE(V33:V78)</f>
+        <f t="shared" si="1"/>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="W79" cm="1">
+        <f t="array" ref="W79">IF(U79, V79, null)</f>
+        <v>9.5367431640625E-4</v>
+      </c>
+      <c r="AC79" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AD79" s="1">
+        <v>2.1457672119140599E-3</v>
+      </c>
+      <c r="AE79" t="b">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF79">
+        <f t="shared" si="3"/>
+        <v>-2.384185791015599E-4</v>
+      </c>
+      <c r="AL79" s="1">
+        <v>6.1988830566406198E-3</v>
+      </c>
+      <c r="AM79" s="1">
+        <v>1.9073486328125E-3</v>
+      </c>
+      <c r="AN79" t="b">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AO79">
+        <f t="shared" si="5"/>
+        <v>1</v>
+      </c>
+      <c r="AP79">
+        <f t="shared" si="6"/>
+        <v>4.2915344238281198E-3</v>
+      </c>
+      <c r="AQ79" cm="1">
+        <f t="array" ref="AQ79">IF(AN79,AP79,null)</f>
+        <v>4.2915344238281198E-3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:43">
+      <c r="V80">
+        <f>AVERAGE(V33:V79)</f>
         <v>1.1247137318486744E-3</v>
       </c>
-      <c r="W79">
-        <f>AVERAGE(W33:W78)</f>
+      <c r="W80">
+        <f>AVERAGE(W33:W79)</f>
         <v>1.7657876014709455E-3</v>
       </c>
-      <c r="AG79">
-        <f>AVERAGE(AG33:AG75)</f>
+      <c r="AG80">
+        <f>AVERAGE(AG33:AG76)</f>
         <v>3.5674483687789305E-3</v>
       </c>
-      <c r="AO79">
-        <f>SUM(AO33:AO78)</f>
+      <c r="AO80">
+        <f>SUM(AO33:AO79)</f>
         <v>20</v>
       </c>
-      <c r="AQ79">
-        <f>AVERAGE(AQ33:AQ78)</f>
+      <c r="AQ80">
+        <f>AVERAGE(AQ33:AQ79)</f>
         <v>7.7605247497558507E-3</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2">
-      <c r="A87">
-        <v>2</v>
-      </c>
-      <c r="B87">
-        <f>(4^A87) *(3^A87)</f>
-        <v>144</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B88">
-        <f t="shared" ref="B88:B89" si="8">4^A88 * 3^A88</f>
-        <v>1728</v>
+        <f>(4^A88) *(3^A88)</f>
+        <v>144</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89">
+        <v>3</v>
+      </c>
+      <c r="B89">
+        <f t="shared" ref="B89:B90" si="8">4^A89 * 3^A89</f>
+        <v>1728</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90">
         <v>4</v>
       </c>
-      <c r="B89">
+      <c r="B90">
         <f t="shared" si="8"/>
         <v>20736</v>
       </c>

</xml_diff>